<commit_message>
finished resytling old RSM executions
</commit_message>
<xml_diff>
--- a/ProbenSpreadsheet.xlsx
+++ b/ProbenSpreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acdcj\Documents\_MasterThesis\DataAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB28A5B5-AB7B-4C0D-967E-380080D3497A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B3D8D4-0967-455F-BC01-D2BBAC456379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51720" yWindow="7155" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51720" yWindow="4785" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Probenübersicht" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
data for new RSM's and plotting done
</commit_message>
<xml_diff>
--- a/ProbenSpreadsheet.xlsx
+++ b/ProbenSpreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acdcj\Documents\_MasterThesis\DataAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B3D8D4-0967-455F-BC01-D2BBAC456379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38E4328-97FE-42FB-B954-4F976B8CDD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51720" yWindow="4785" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51720" yWindow="7155" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Probenübersicht" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1754" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1758" uniqueCount="316">
   <si>
     <t>Id</t>
   </si>
@@ -12295,7 +12295,9 @@
         <v>144</v>
       </c>
       <c r="AB171" s="255"/>
-      <c r="AC171" s="255"/>
+      <c r="AC171" s="255" t="s">
+        <v>144</v>
+      </c>
       <c r="AD171" s="21"/>
     </row>
     <row r="172" spans="1:30" s="24" customFormat="1" x14ac:dyDescent="0.55000000000000004">
@@ -12408,7 +12410,7 @@
       </c>
       <c r="AB173" s="255"/>
       <c r="AC173" s="255" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="AD173" s="21"/>
     </row>
@@ -12975,7 +12977,9 @@
         <v>144</v>
       </c>
       <c r="AB183" s="258"/>
-      <c r="AC183" s="258"/>
+      <c r="AC183" s="258" t="s">
+        <v>144</v>
+      </c>
       <c r="AD183" s="25"/>
     </row>
     <row r="184" spans="1:30" s="175" customFormat="1" x14ac:dyDescent="0.55000000000000004">
@@ -13201,7 +13205,9 @@
         <v>144</v>
       </c>
       <c r="AB187" s="255"/>
-      <c r="AC187" s="255"/>
+      <c r="AC187" s="255" t="s">
+        <v>144</v>
+      </c>
       <c r="AD187" s="21"/>
     </row>
     <row r="188" spans="1:30" s="24" customFormat="1" x14ac:dyDescent="0.55000000000000004">
@@ -13315,7 +13321,7 @@
       </c>
       <c r="AB189" s="255"/>
       <c r="AC189" s="255" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="AD189" s="21"/>
     </row>
@@ -13429,7 +13435,9 @@
         <v>144</v>
       </c>
       <c r="AB191" s="258"/>
-      <c r="AC191" s="258"/>
+      <c r="AC191" s="258" t="s">
+        <v>144</v>
+      </c>
       <c r="AD191" s="25"/>
     </row>
     <row r="192" spans="1:30" s="175" customFormat="1" x14ac:dyDescent="0.55000000000000004">
@@ -13543,7 +13551,7 @@
       </c>
       <c r="AB193" s="258"/>
       <c r="AC193" s="258" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="AD193" s="25"/>
     </row>

</xml_diff>